<commit_message>
bugfix: calculate leadership rate correctly
</commit_message>
<xml_diff>
--- a/unit_stats_last_30_days.xlsx
+++ b/unit_stats_last_30_days.xlsx
@@ -476,7 +476,7 @@
         <v>460</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8152173913043478</v>
+        <v>0.7913043478260869</v>
       </c>
       <c r="E2" t="n">
         <v>4.238663484486874</v>
@@ -510,7 +510,7 @@
         <v>109</v>
       </c>
       <c r="D3" t="n">
-        <v>3.440366972477064</v>
+        <v>0.6880733944954128</v>
       </c>
       <c r="E3" t="n">
         <v>6.163636363636364</v>
@@ -544,7 +544,7 @@
         <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>13.39285714285714</v>
+        <v>0.8214285714285714</v>
       </c>
       <c r="E4" t="n">
         <v>5.72</v>
@@ -612,7 +612,7 @@
         <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>125</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -646,7 +646,7 @@
         <v>483</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7763975155279503</v>
+        <v>0.7867494824016563</v>
       </c>
       <c r="E7" t="n">
         <v>4.8165548098434</v>
@@ -680,7 +680,7 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>187.5</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>5</v>
@@ -712,7 +712,7 @@
         <v>153</v>
       </c>
       <c r="D9" t="n">
-        <v>2.450980392156863</v>
+        <v>0.7450980392156863</v>
       </c>
       <c r="E9" t="n">
         <v>5.577464788732394</v>
@@ -746,7 +746,7 @@
         <v>305</v>
       </c>
       <c r="D10" t="n">
-        <v>1.229508196721312</v>
+        <v>0.7508196721311475</v>
       </c>
       <c r="E10" t="n">
         <v>4.44</v>
@@ -780,7 +780,7 @@
         <v>461</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8134490238611713</v>
+        <v>0.7722342733188721</v>
       </c>
       <c r="E11" t="n">
         <v>4.949029126213592</v>
@@ -814,7 +814,7 @@
         <v>49</v>
       </c>
       <c r="D12" t="n">
-        <v>7.653061224489796</v>
+        <v>0.8367346938775511</v>
       </c>
       <c r="E12" t="n">
         <v>6.422222222222222</v>
@@ -848,7 +848,7 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
@@ -878,7 +878,7 @@
         <v>34</v>
       </c>
       <c r="D14" t="n">
-        <v>11.02941176470588</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
         <v>17.41666666666667</v>
@@ -912,7 +912,7 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
@@ -942,7 +942,7 @@
         <v>94</v>
       </c>
       <c r="D16" t="n">
-        <v>3.98936170212766</v>
+        <v>0.01063829787234043</v>
       </c>
       <c r="E16" t="n">
         <v>6.338983050847458</v>
@@ -976,7 +976,7 @@
         <v>44</v>
       </c>
       <c r="D17" t="n">
-        <v>8.522727272727273</v>
+        <v>0.02272727272727273</v>
       </c>
       <c r="E17" t="n">
         <v>8.727272727272727</v>
@@ -1010,7 +1010,7 @@
         <v>67</v>
       </c>
       <c r="D18" t="n">
-        <v>5.597014925373134</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
         <v>7.804878048780488</v>
@@ -1044,7 +1044,7 @@
         <v>61</v>
       </c>
       <c r="D19" t="n">
-        <v>6.147540983606557</v>
+        <v>0.01639344262295082</v>
       </c>
       <c r="E19" t="n">
         <v>7.822222222222222</v>
@@ -1078,7 +1078,7 @@
         <v>34</v>
       </c>
       <c r="D20" t="n">
-        <v>11.02941176470588</v>
+        <v>0.02941176470588235</v>
       </c>
       <c r="E20" t="n">
         <v>6.478260869565218</v>
@@ -1112,7 +1112,7 @@
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -1142,7 +1142,7 @@
         <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>41.66666666666666</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
         <v>104.5</v>
@@ -1176,7 +1176,7 @@
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
@@ -1206,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
@@ -1236,7 +1236,7 @@
         <v>8</v>
       </c>
       <c r="D25" t="n">
-        <v>46.875</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
         <v>15</v>
@@ -1270,7 +1270,7 @@
         <v>34</v>
       </c>
       <c r="D26" t="n">
-        <v>11.02941176470588</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
         <v>8.625</v>
@@ -1304,7 +1304,7 @@
         <v>327</v>
       </c>
       <c r="D27" t="n">
-        <v>1.146788990825688</v>
+        <v>0.7522935779816514</v>
       </c>
       <c r="E27" t="n">
         <v>4.384057971014493</v>
@@ -1338,7 +1338,7 @@
         <v>137</v>
       </c>
       <c r="D28" t="n">
-        <v>2.737226277372263</v>
+        <v>0.8394160583941606</v>
       </c>
       <c r="E28" t="n">
         <v>5.350746268656716</v>
@@ -1372,7 +1372,7 @@
         <v>223</v>
       </c>
       <c r="D29" t="n">
-        <v>1.681614349775785</v>
+        <v>0.7713004484304933</v>
       </c>
       <c r="E29" t="n">
         <v>5.306930693069307</v>
@@ -1406,7 +1406,7 @@
         <v>178</v>
       </c>
       <c r="D30" t="n">
-        <v>2.106741573033708</v>
+        <v>0.7808988764044944</v>
       </c>
       <c r="E30" t="n">
         <v>4.993548387096774</v>
@@ -1440,7 +1440,7 @@
         <v>345</v>
       </c>
       <c r="D31" t="n">
-        <v>1.08695652173913</v>
+        <v>0.8463768115942029</v>
       </c>
       <c r="E31" t="n">
         <v>4.564102564102564</v>
@@ -1474,7 +1474,7 @@
         <v>265</v>
       </c>
       <c r="D32" t="n">
-        <v>1.415094339622641</v>
+        <v>0.8075471698113208</v>
       </c>
       <c r="E32" t="n">
         <v>4.298755186721992</v>
@@ -1508,7 +1508,7 @@
         <v>385</v>
       </c>
       <c r="D33" t="n">
-        <v>0.974025974025974</v>
+        <v>0.7610389610389611</v>
       </c>
       <c r="E33" t="n">
         <v>4.716867469879518</v>
@@ -1542,7 +1542,7 @@
         <v>116</v>
       </c>
       <c r="D34" t="n">
-        <v>3.232758620689655</v>
+        <v>0.8189655172413793</v>
       </c>
       <c r="E34" t="n">
         <v>4.801980198019802</v>
@@ -1576,7 +1576,7 @@
         <v>167</v>
       </c>
       <c r="D35" t="n">
-        <v>2.245508982035928</v>
+        <v>0.7844311377245509</v>
       </c>
       <c r="E35" t="n">
         <v>4.414965986394558</v>
@@ -1610,7 +1610,7 @@
         <v>87</v>
       </c>
       <c r="D36" t="n">
-        <v>4.310344827586207</v>
+        <v>0.7241379310344828</v>
       </c>
       <c r="E36" t="n">
         <v>6.105263157894737</v>
@@ -1644,7 +1644,7 @@
         <v>293</v>
       </c>
       <c r="D37" t="n">
-        <v>1.279863481228669</v>
+        <v>0.8191126279863481</v>
       </c>
       <c r="E37" t="n">
         <v>4.523297491039426</v>
@@ -1678,7 +1678,7 @@
         <v>374</v>
       </c>
       <c r="D38" t="n">
-        <v>1.002673796791444</v>
+        <v>0.7727272727272727</v>
       </c>
       <c r="E38" t="n">
         <v>4.358730158730158</v>
@@ -1712,7 +1712,7 @@
         <v>75</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="E39" t="n">
         <v>4.82089552238806</v>
@@ -1746,7 +1746,7 @@
         <v>104</v>
       </c>
       <c r="D40" t="n">
-        <v>3.605769230769231</v>
+        <v>0.6057692307692307</v>
       </c>
       <c r="E40" t="n">
         <v>5.494252873563219</v>
@@ -1780,7 +1780,7 @@
         <v>307</v>
       </c>
       <c r="D41" t="n">
-        <v>1.221498371335505</v>
+        <v>0.8078175895765473</v>
       </c>
       <c r="E41" t="n">
         <v>4.589473684210526</v>
@@ -1814,7 +1814,7 @@
         <v>129</v>
       </c>
       <c r="D42" t="n">
-        <v>2.906976744186046</v>
+        <v>0.813953488372093</v>
       </c>
       <c r="E42" t="n">
         <v>5.411764705882353</v>
@@ -1848,7 +1848,7 @@
         <v>285</v>
       </c>
       <c r="D43" t="n">
-        <v>1.315789473684211</v>
+        <v>0.8035087719298246</v>
       </c>
       <c r="E43" t="n">
         <v>4</v>
@@ -1882,7 +1882,7 @@
         <v>270</v>
       </c>
       <c r="D44" t="n">
-        <v>1.388888888888889</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E44" t="n">
         <v>4.970588235294118</v>
@@ -1916,7 +1916,7 @@
         <v>192</v>
       </c>
       <c r="D45" t="n">
-        <v>1.953125</v>
+        <v>0.78125</v>
       </c>
       <c r="E45" t="n">
         <v>4.780346820809249</v>
@@ -1950,7 +1950,7 @@
         <v>196</v>
       </c>
       <c r="D46" t="n">
-        <v>1.913265306122449</v>
+        <v>0.8367346938775511</v>
       </c>
       <c r="E46" t="n">
         <v>4.211956521739131</v>
@@ -1984,7 +1984,7 @@
         <v>111</v>
       </c>
       <c r="D47" t="n">
-        <v>3.378378378378379</v>
+        <v>0.8288288288288288</v>
       </c>
       <c r="E47" t="n">
         <v>4.793814432989691</v>
@@ -2018,7 +2018,7 @@
         <v>157</v>
       </c>
       <c r="D48" t="n">
-        <v>2.388535031847134</v>
+        <v>0.802547770700637</v>
       </c>
       <c r="E48" t="n">
         <v>5.155555555555556</v>
@@ -2052,7 +2052,7 @@
         <v>104</v>
       </c>
       <c r="D49" t="n">
-        <v>3.605769230769231</v>
+        <v>0.6730769230769231</v>
       </c>
       <c r="E49" t="n">
         <v>6.27906976744186</v>
@@ -2086,7 +2086,7 @@
         <v>202</v>
       </c>
       <c r="D50" t="n">
-        <v>1.856435643564357</v>
+        <v>0.806930693069307</v>
       </c>
       <c r="E50" t="n">
         <v>5.26775956284153</v>
@@ -2120,7 +2120,7 @@
         <v>188</v>
       </c>
       <c r="D51" t="n">
-        <v>1.99468085106383</v>
+        <v>0.824468085106383</v>
       </c>
       <c r="E51" t="n">
         <v>5.0625</v>
@@ -2154,7 +2154,7 @@
         <v>220</v>
       </c>
       <c r="D52" t="n">
-        <v>1.704545454545455</v>
+        <v>0.8727272727272727</v>
       </c>
       <c r="E52" t="n">
         <v>5.371428571428571</v>
@@ -2188,7 +2188,7 @@
         <v>146</v>
       </c>
       <c r="D53" t="n">
-        <v>2.568493150684931</v>
+        <v>0.7534246575342466</v>
       </c>
       <c r="E53" t="n">
         <v>5.1171875</v>
@@ -2222,7 +2222,7 @@
         <v>75</v>
       </c>
       <c r="D54" t="n">
-        <v>5</v>
+        <v>0.8933333333333333</v>
       </c>
       <c r="E54" t="n">
         <v>5.410958904109589</v>
@@ -2256,7 +2256,7 @@
         <v>261</v>
       </c>
       <c r="D55" t="n">
-        <v>1.436781609195402</v>
+        <v>0.7241379310344828</v>
       </c>
       <c r="E55" t="n">
         <v>4.645739910313901</v>
@@ -2290,7 +2290,7 @@
         <v>321</v>
       </c>
       <c r="D56" t="n">
-        <v>1.168224299065421</v>
+        <v>0.7757009345794392</v>
       </c>
       <c r="E56" t="n">
         <v>4.11437908496732</v>
@@ -2324,7 +2324,7 @@
         <v>177</v>
       </c>
       <c r="D57" t="n">
-        <v>2.11864406779661</v>
+        <v>0.847457627118644</v>
       </c>
       <c r="E57" t="n">
         <v>5.221518987341772</v>
@@ -2358,7 +2358,7 @@
         <v>199</v>
       </c>
       <c r="D58" t="n">
-        <v>1.884422110552764</v>
+        <v>0.7788944723618091</v>
       </c>
       <c r="E58" t="n">
         <v>4.681564245810056</v>
@@ -2392,7 +2392,7 @@
         <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E59" t="n">
         <v>0</v>
@@ -2422,7 +2422,7 @@
         <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
@@ -2452,7 +2452,7 @@
         <v>1</v>
       </c>
       <c r="D61" t="n">
-        <v>375</v>
+        <v>1</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
@@ -2482,7 +2482,7 @@
         <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>375</v>
+        <v>1</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
@@ -2512,7 +2512,7 @@
         <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>125</v>
+        <v>1</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
@@ -2542,7 +2542,7 @@
         <v>13</v>
       </c>
       <c r="D64" t="n">
-        <v>28.84615384615385</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="E64" t="n">
         <v>0.3846153846153846</v>
@@ -2576,7 +2576,7 @@
         <v>14</v>
       </c>
       <c r="D65" t="n">
-        <v>26.78571428571428</v>
+        <v>0.7857142857142857</v>
       </c>
       <c r="E65" t="n">
         <v>0</v>
@@ -2606,7 +2606,7 @@
         <v>9</v>
       </c>
       <c r="D66" t="n">
-        <v>41.66666666666666</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
@@ -2640,7 +2640,7 @@
         <v>1</v>
       </c>
       <c r="D67" t="n">
-        <v>375</v>
+        <v>1</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
@@ -2670,7 +2670,7 @@
         <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>375</v>
+        <v>1</v>
       </c>
       <c r="E68" t="n">
         <v>1</v>
@@ -2700,7 +2700,7 @@
         <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>375</v>
+        <v>1</v>
       </c>
       <c r="E69" t="n">
         <v>0</v>
@@ -2730,7 +2730,7 @@
         <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>375</v>
+        <v>1</v>
       </c>
       <c r="E70" t="n">
         <v>0</v>
@@ -2760,7 +2760,7 @@
         <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>375</v>
+        <v>1</v>
       </c>
       <c r="E71" t="n">
         <v>0</v>
@@ -2790,7 +2790,7 @@
         <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>375</v>
+        <v>1</v>
       </c>
       <c r="E72" t="n">
         <v>0</v>
@@ -2820,7 +2820,7 @@
         <v>5</v>
       </c>
       <c r="D73" t="n">
-        <v>75</v>
+        <v>0.6</v>
       </c>
       <c r="E73" t="n">
         <v>0</v>
@@ -2854,7 +2854,7 @@
         <v>8</v>
       </c>
       <c r="D74" t="n">
-        <v>46.875</v>
+        <v>0.75</v>
       </c>
       <c r="E74" t="n">
         <v>0</v>
@@ -2888,7 +2888,7 @@
         <v>6</v>
       </c>
       <c r="D75" t="n">
-        <v>62.5</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="E75" t="n">
         <v>13.66666666666667</v>
@@ -2922,7 +2922,7 @@
         <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="E76" t="n">
         <v>49</v>
@@ -2956,7 +2956,7 @@
         <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E77" t="n">
         <v>0</v>
@@ -2990,7 +2990,7 @@
         <v>18</v>
       </c>
       <c r="D78" t="n">
-        <v>20.83333333333333</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="E78" t="n">
         <v>0</v>
@@ -3024,7 +3024,7 @@
         <v>88</v>
       </c>
       <c r="D79" t="n">
-        <v>4.261363636363637</v>
+        <v>0.7840909090909091</v>
       </c>
       <c r="E79" t="n">
         <v>13.25</v>
@@ -3058,7 +3058,7 @@
         <v>2</v>
       </c>
       <c r="D80" t="n">
-        <v>187.5</v>
+        <v>0</v>
       </c>
       <c r="E80" t="n">
         <v>28</v>
@@ -3092,7 +3092,7 @@
         <v>41</v>
       </c>
       <c r="D81" t="n">
-        <v>9.146341463414634</v>
+        <v>0.8536585365853658</v>
       </c>
       <c r="E81" t="n">
         <v>12.08108108108108</v>
@@ -3126,7 +3126,7 @@
         <v>37</v>
       </c>
       <c r="D82" t="n">
-        <v>10.13513513513514</v>
+        <v>0.7297297297297297</v>
       </c>
       <c r="E82" t="n">
         <v>7.666666666666667</v>
@@ -3160,7 +3160,7 @@
         <v>91</v>
       </c>
       <c r="D83" t="n">
-        <v>4.12087912087912</v>
+        <v>0.04395604395604396</v>
       </c>
       <c r="E83" t="n">
         <v>6.376623376623376</v>
@@ -3194,7 +3194,7 @@
         <v>8</v>
       </c>
       <c r="D84" t="n">
-        <v>46.875</v>
+        <v>0</v>
       </c>
       <c r="E84" t="n">
         <v>12.8</v>
@@ -3228,7 +3228,7 @@
         <v>2</v>
       </c>
       <c r="D85" t="n">
-        <v>187.5</v>
+        <v>0</v>
       </c>
       <c r="E85" t="n">
         <v>0</v>
@@ -3258,7 +3258,7 @@
         <v>4</v>
       </c>
       <c r="D86" t="n">
-        <v>93.75</v>
+        <v>0</v>
       </c>
       <c r="E86" t="n">
         <v>0</v>
@@ -3292,7 +3292,7 @@
         <v>235</v>
       </c>
       <c r="D87" t="n">
-        <v>1.595744680851064</v>
+        <v>0.3106382978723404</v>
       </c>
       <c r="E87" t="n">
         <v>5.219251336898396</v>
@@ -3326,7 +3326,7 @@
         <v>250</v>
       </c>
       <c r="D88" t="n">
-        <v>1.5</v>
+        <v>0.312</v>
       </c>
       <c r="E88" t="n">
         <v>4.680628272251309</v>
@@ -3360,7 +3360,7 @@
         <v>98</v>
       </c>
       <c r="D89" t="n">
-        <v>3.826530612244898</v>
+        <v>0.4183673469387755</v>
       </c>
       <c r="E89" t="n">
         <v>5.618421052631579</v>
@@ -3394,7 +3394,7 @@
         <v>159</v>
       </c>
       <c r="D90" t="n">
-        <v>2.358490566037736</v>
+        <v>0.4716981132075472</v>
       </c>
       <c r="E90" t="n">
         <v>5.590163934426229</v>
@@ -3428,7 +3428,7 @@
         <v>96</v>
       </c>
       <c r="D91" t="n">
-        <v>3.90625</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="E91" t="n">
         <v>5.736111111111111</v>
@@ -3462,7 +3462,7 @@
         <v>194</v>
       </c>
       <c r="D92" t="n">
-        <v>1.93298969072165</v>
+        <v>0.4175257731958763</v>
       </c>
       <c r="E92" t="n">
         <v>5.272727272727272</v>
@@ -3496,7 +3496,7 @@
         <v>264</v>
       </c>
       <c r="D93" t="n">
-        <v>1.420454545454545</v>
+        <v>0.3371212121212121</v>
       </c>
       <c r="E93" t="n">
         <v>5.477832512315271</v>
@@ -3530,7 +3530,7 @@
         <v>183</v>
       </c>
       <c r="D94" t="n">
-        <v>2.049180327868852</v>
+        <v>0.3825136612021858</v>
       </c>
       <c r="E94" t="n">
         <v>7.479338842975206</v>
@@ -3564,7 +3564,7 @@
         <v>110</v>
       </c>
       <c r="D95" t="n">
-        <v>3.409090909090909</v>
+        <v>0.3727272727272727</v>
       </c>
       <c r="E95" t="n">
         <v>6.565789473684211</v>
@@ -3598,7 +3598,7 @@
         <v>168</v>
       </c>
       <c r="D96" t="n">
-        <v>2.232142857142857</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="E96" t="n">
         <v>7</v>
@@ -3632,7 +3632,7 @@
         <v>222</v>
       </c>
       <c r="D97" t="n">
-        <v>1.689189189189189</v>
+        <v>0.3558558558558558</v>
       </c>
       <c r="E97" t="n">
         <v>5.927272727272728</v>
@@ -3666,7 +3666,7 @@
         <v>1</v>
       </c>
       <c r="D98" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E98" t="n">
         <v>0</v>
@@ -3696,7 +3696,7 @@
         <v>2</v>
       </c>
       <c r="D99" t="n">
-        <v>187.5</v>
+        <v>0</v>
       </c>
       <c r="E99" t="n">
         <v>2.5</v>
@@ -3726,7 +3726,7 @@
         <v>1</v>
       </c>
       <c r="D100" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E100" t="n">
         <v>0</v>
@@ -3756,7 +3756,7 @@
         <v>367</v>
       </c>
       <c r="D101" t="n">
-        <v>1.021798365122616</v>
+        <v>0.444141689373297</v>
       </c>
       <c r="E101" t="n">
         <v>7.042307692307692</v>
@@ -3790,7 +3790,7 @@
         <v>334</v>
       </c>
       <c r="D102" t="n">
-        <v>1.122754491017964</v>
+        <v>0.4491017964071856</v>
       </c>
       <c r="E102" t="n">
         <v>7.254385964912281</v>
@@ -3824,7 +3824,7 @@
         <v>254</v>
       </c>
       <c r="D103" t="n">
-        <v>1.476377952755906</v>
+        <v>0.3740157480314961</v>
       </c>
       <c r="E103" t="n">
         <v>7.791411042944786</v>
@@ -3858,7 +3858,7 @@
         <v>142</v>
       </c>
       <c r="D104" t="n">
-        <v>2.640845070422535</v>
+        <v>0.3732394366197183</v>
       </c>
       <c r="E104" t="n">
         <v>8.065217391304348</v>
@@ -3892,7 +3892,7 @@
         <v>51</v>
       </c>
       <c r="D105" t="n">
-        <v>7.352941176470588</v>
+        <v>0.392156862745098</v>
       </c>
       <c r="E105" t="n">
         <v>8.058823529411764</v>
@@ -3926,7 +3926,7 @@
         <v>184</v>
       </c>
       <c r="D106" t="n">
-        <v>2.03804347826087</v>
+        <v>0.4076086956521739</v>
       </c>
       <c r="E106" t="n">
         <v>7.215277777777778</v>
@@ -3960,7 +3960,7 @@
         <v>156</v>
       </c>
       <c r="D107" t="n">
-        <v>2.403846153846154</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="E107" t="n">
         <v>7.832</v>
@@ -3994,7 +3994,7 @@
         <v>161</v>
       </c>
       <c r="D108" t="n">
-        <v>2.329192546583851</v>
+        <v>0.453416149068323</v>
       </c>
       <c r="E108" t="n">
         <v>7.798245614035087</v>
@@ -4028,7 +4028,7 @@
         <v>92</v>
       </c>
       <c r="D109" t="n">
-        <v>4.076086956521739</v>
+        <v>0</v>
       </c>
       <c r="E109" t="n">
         <v>8.708333333333334</v>
@@ -4062,7 +4062,7 @@
         <v>42</v>
       </c>
       <c r="D110" t="n">
-        <v>8.928571428571429</v>
+        <v>0</v>
       </c>
       <c r="E110" t="n">
         <v>19.36363636363636</v>
@@ -4096,7 +4096,7 @@
         <v>60</v>
       </c>
       <c r="D111" t="n">
-        <v>6.25</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="E111" t="n">
         <v>19</v>
@@ -4130,7 +4130,7 @@
         <v>4</v>
       </c>
       <c r="D112" t="n">
-        <v>93.75</v>
+        <v>0</v>
       </c>
       <c r="E112" t="n">
         <v>27.5</v>
@@ -4164,7 +4164,7 @@
         <v>4</v>
       </c>
       <c r="D113" t="n">
-        <v>93.75</v>
+        <v>0</v>
       </c>
       <c r="E113" t="n">
         <v>26.33333333333333</v>
@@ -4198,7 +4198,7 @@
         <v>4</v>
       </c>
       <c r="D114" t="n">
-        <v>93.75</v>
+        <v>0</v>
       </c>
       <c r="E114" t="n">
         <v>16.5</v>
@@ -4232,7 +4232,7 @@
         <v>1</v>
       </c>
       <c r="D115" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="n">
@@ -4262,7 +4262,7 @@
         <v>3</v>
       </c>
       <c r="D116" t="n">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="E116" t="n">
         <v>5.666666666666667</v>
@@ -4296,7 +4296,7 @@
         <v>13</v>
       </c>
       <c r="D117" t="n">
-        <v>28.84615384615385</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="E117" t="n">
         <v>0</v>
@@ -4326,7 +4326,7 @@
         <v>6</v>
       </c>
       <c r="D118" t="n">
-        <v>62.5</v>
+        <v>0</v>
       </c>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="n">
@@ -4356,7 +4356,7 @@
         <v>123</v>
       </c>
       <c r="D119" t="n">
-        <v>3.048780487804878</v>
+        <v>0.2520325203252032</v>
       </c>
       <c r="E119" t="n">
         <v>7.645569620253164</v>
@@ -4390,7 +4390,7 @@
         <v>2</v>
       </c>
       <c r="D120" t="n">
-        <v>187.5</v>
+        <v>0</v>
       </c>
       <c r="E120" t="n">
         <v>20</v>
@@ -4424,7 +4424,7 @@
         <v>27</v>
       </c>
       <c r="D121" t="n">
-        <v>13.88888888888889</v>
+        <v>0.03703703703703703</v>
       </c>
       <c r="E121" t="n">
         <v>13.85714285714286</v>
@@ -4458,7 +4458,7 @@
         <v>66</v>
       </c>
       <c r="D122" t="n">
-        <v>5.681818181818182</v>
+        <v>0</v>
       </c>
       <c r="E122" t="n">
         <v>10.87878787878788</v>
@@ -4492,7 +4492,7 @@
         <v>3</v>
       </c>
       <c r="D123" t="n">
-        <v>125</v>
+        <v>1</v>
       </c>
       <c r="E123" t="n">
         <v>0</v>
@@ -4522,7 +4522,7 @@
         <v>34</v>
       </c>
       <c r="D124" t="n">
-        <v>11.02941176470588</v>
+        <v>0</v>
       </c>
       <c r="E124" t="n">
         <v>11.25</v>
@@ -4556,7 +4556,7 @@
         <v>2</v>
       </c>
       <c r="D125" t="n">
-        <v>187.5</v>
+        <v>0</v>
       </c>
       <c r="E125" t="n">
         <v>0</v>
@@ -4586,7 +4586,7 @@
         <v>6</v>
       </c>
       <c r="D126" t="n">
-        <v>62.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E126" t="n">
         <v>0</v>

</xml_diff>